<commit_message>
Change ConsumeForcast Excell File
</commit_message>
<xml_diff>
--- a/src/Datiss.Budget.Web/wwwroot/excel/ConsumeForcastImport.xlsx
+++ b/src/Datiss.Budget.Web/wwwroot/excel/ConsumeForcastImport.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24816"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FinalDatiss\Datiss\datiss.budget\src\Datiss.Budget.Web\wwwroot\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Datiss\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FA9ABBB-3B82-415A-8FE7-DCB977B03EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70FBAD00-81F0-4666-B897-1A4A58E2E8A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3270" yWindow="5985" windowWidth="15465" windowHeight="11055" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,24 +25,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>Column1</t>
-  </si>
-  <si>
-    <t>Column2</t>
-  </si>
-  <si>
-    <t>Column3</t>
-  </si>
-  <si>
-    <t>Column4</t>
-  </si>
-  <si>
-    <t>Column5</t>
-  </si>
-  <si>
-    <t>Column6</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+  <si>
+    <t>سال</t>
+  </si>
+  <si>
+    <t>سازمان</t>
+  </si>
+  <si>
+    <t>کاربری</t>
+  </si>
+  <si>
+    <t>طبقه مصرف</t>
+  </si>
+  <si>
+    <t>توزیع تعدادی</t>
+  </si>
+  <si>
+    <t>توزیع آحادی</t>
+  </si>
+  <si>
+    <t>توزیع مصرف</t>
+  </si>
+  <si>
+    <t>میانگین مصرف</t>
   </si>
 </sst>
 </file>
@@ -86,13 +92,47 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="10">
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -106,15 +146,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:F3" totalsRowShown="0">
-  <autoFilter ref="A1:F3" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Column1"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Column2"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Column3"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Column4"/>
-    <tableColumn id="5" xr3:uid="{A66BFD00-0347-49B8-BF8A-44E031E4CF50}" name="Column5"/>
-    <tableColumn id="6" xr3:uid="{156DFAC3-C12B-4E27-BB8A-FB54A53C3CD9}" name="Column6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:H3" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+  <autoFilter ref="A1:H3" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="سال" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="سازمان" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="کاربری" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="طبقه مصرف" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{A66BFD00-0347-49B8-BF8A-44E031E4CF50}" name="توزیع تعدادی" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{3CC44A50-C07F-4ABB-AEB7-802FA719BE66}" name="توزیع آحادی" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{DB09B25D-7B6F-41D7-B7B9-F28F58BDDC8E}" name="توزیع مصرف" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{156DFAC3-C12B-4E27-BB8A-FB54A53C3CD9}" name="میانگین مصرف" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -383,70 +425,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="4" width="11" customWidth="1"/>
+    <col min="1" max="8" width="13" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>4</v>
-      </c>
-      <c r="C2">
-        <v>4</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>25</v>
-      </c>
-      <c r="F2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3">
-        <v>4</v>
-      </c>
-      <c r="C3">
-        <v>5</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>47</v>
-      </c>
-      <c r="F3">
-        <v>9</v>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>